<commit_message>
Complete FEI signal validation matrix
</commit_message>
<xml_diff>
--- a/docs/signal_availability_matrix.xlsx
+++ b/docs/signal_availability_matrix.xlsx
@@ -8,12 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/haneuljang/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D212B439-869F-B347-AE65-897B394CF386}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F253B4F2-62A2-5248-AE1B-DB13A59C31FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5180" yWindow="1800" windowWidth="28040" windowHeight="17440" xr2:uid="{29318AA6-4BD7-6244-B5A3-8C80AA045784}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="21360" activeTab="3" xr2:uid="{29318AA6-4BD7-6244-B5A3-8C80AA045784}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="FEI Signal Validation" sheetId="1" r:id="rId1"/>
+    <sheet name="DSI Signal Validation" sheetId="2" r:id="rId2"/>
+    <sheet name="VEI Signal Validation" sheetId="3" r:id="rId3"/>
+    <sheet name="Signal Gap Analysis" sheetId="4" r:id="rId4"/>
+    <sheet name="OEM Limitation Summary" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -35,9 +39,288 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="86">
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Signal</t>
+  </si>
+  <si>
+    <t>Required for Full FEI</t>
+  </si>
+  <si>
+    <t>Final Status</t>
+  </si>
+  <si>
+    <t>Business Impact</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Engine RPM</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Available</t>
+  </si>
+  <si>
+    <t>Engine Load</t>
+  </si>
+  <si>
+    <t>Not Available</t>
+  </si>
+  <si>
+    <t>Fuel Rate</t>
+  </si>
+  <si>
+    <t>Engine Hours</t>
+  </si>
+  <si>
+    <t>Distance / Odometer</t>
+  </si>
+  <si>
+    <t>Torque</t>
+  </si>
+  <si>
+    <t>Preferred</t>
+  </si>
+  <si>
+    <t>Vehicle Speed</t>
+  </si>
+  <si>
+    <t>Fuel Used Counter</t>
+  </si>
+  <si>
+    <t>Limits driver demand analysis</t>
+  </si>
+  <si>
+    <t>Advanced</t>
+  </si>
+  <si>
+    <t>Priority</t>
+  </si>
+  <si>
+    <t>GeoTab Diagnostic Exists</t>
+  </si>
+  <si>
+    <t>Timestamp</t>
+  </si>
+  <si>
+    <t>Mandatory</t>
+  </si>
+  <si>
+    <t>Vehicle ID</t>
+  </si>
+  <si>
+    <t>Full FEI cannot be implemented</t>
+  </si>
+  <si>
+    <t>Partial</t>
+  </si>
+  <si>
+    <t>Cruise Status</t>
+  </si>
+  <si>
+    <t>PTO Status</t>
+  </si>
+  <si>
+    <t>Coolant Temperature</t>
+  </si>
+  <si>
+    <t>Available operational signal</t>
+  </si>
+  <si>
+    <t>Vehicle Count With Data</t>
+  </si>
+  <si>
+    <t>Required for all time-series calculations</t>
+  </si>
+  <si>
+    <t>Available from StatusData</t>
+  </si>
+  <si>
+    <t>VIN</t>
+  </si>
+  <si>
+    <t>Vehicle identification</t>
+  </si>
+  <si>
+    <t>Available through GeoTab</t>
+  </si>
+  <si>
+    <t>Vehicle aggregation key</t>
+  </si>
+  <si>
+    <t>Core FEI parameter</t>
+  </si>
+  <si>
+    <t>Engine Speed diagnostic available</t>
+  </si>
+  <si>
+    <t>No StatusData observed on DHL fleet</t>
+  </si>
+  <si>
+    <t>Supports utilization normalization</t>
+  </si>
+  <si>
+    <t>Supports fuel-efficiency calculation</t>
+  </si>
+  <si>
+    <t>Odometer available</t>
+  </si>
+  <si>
+    <t>Supports driving behavior analysis</t>
+  </si>
+  <si>
+    <t>Useful for FEI-Lite</t>
+  </si>
+  <si>
+    <t>Accelerator Pedal Position (APS)</t>
+  </si>
+  <si>
+    <t>No DHL StatusData observed</t>
+  </si>
+  <si>
+    <t>Supports fuel-efficiency calculations</t>
+  </si>
+  <si>
+    <t>Total Fuel Used available</t>
+  </si>
+  <si>
+    <t>Idle Status</t>
+  </si>
+  <si>
+    <t>Supports idle efficiency analysis</t>
+  </si>
+  <si>
+    <t>Idle metrics available</t>
+  </si>
+  <si>
+    <t>Optional FEI enhancement</t>
+  </si>
+  <si>
+    <t>Improves engine work modeling</t>
+  </si>
+  <si>
+    <t>Boost Pressure</t>
+  </si>
+  <si>
+    <t>Future FEI enhancement</t>
+  </si>
+  <si>
+    <t>Not observed</t>
+  </si>
+  <si>
+    <t>Engine health context</t>
+  </si>
+  <si>
+    <t>Rail Pressure</t>
+  </si>
+  <si>
+    <t>Intake Temperature</t>
+  </si>
+  <si>
+    <t>Requires additional validation</t>
+  </si>
+  <si>
+    <t>Not observed in diagnostic mapping or pilot data</t>
+  </si>
+  <si>
+    <t>PTO Fuel Used diagnostic detected</t>
+  </si>
+  <si>
+    <t>Boost-related diagnostics detected</t>
+  </si>
+  <si>
+    <t>Cruise control enabled and Cruise control active observed in DHL pilot data</t>
+  </si>
+  <si>
+    <t>DHL Pilot
+ Data Available</t>
+  </si>
+  <si>
+    <t>FEI Validation Summary</t>
+  </si>
+  <si>
+    <t>Result</t>
+  </si>
+  <si>
+    <t>Critical Signals Available</t>
+  </si>
+  <si>
+    <t>RPM, Distance/Odometer</t>
+  </si>
+  <si>
+    <t>Operational Signals Available</t>
+  </si>
+  <si>
+    <t>Fuel Used, Vehicle Speed, Idle Status, Cruise Status, Coolant Temperature</t>
+  </si>
+  <si>
+    <t>Critical Signals Missing</t>
+  </si>
+  <si>
+    <t>Engine Load, Fuel Rate</t>
+  </si>
+  <si>
+    <t>High-Value Signals Missing</t>
+  </si>
+  <si>
+    <t>Additional Missing Signals</t>
+  </si>
+  <si>
+    <t>APS</t>
+  </si>
+  <si>
+    <t>Full FEI Feasible</t>
+  </si>
+  <si>
+    <t>FEI-Lite Feasible</t>
+  </si>
+  <si>
+    <t>Key Findings</t>
+  </si>
+  <si>
+    <t>Final Conclusion</t>
+  </si>
+  <si>
+    <t>Required FEI Signals Evaluated | 19</t>
+  </si>
+  <si>
+    <t>Validation Result
+The DHL Hyundai pilot fleet does not currently provide the critical telemetry signals required for Full FEI implementation.
+Missing Critical Signals:
+- Engine Load
+- Fuel Rate
+Missing High-Value Signals:
+- Torque
+- Accelerator Pedal Position (APS)
+Therefore, Full FEI implementation is not currently feasible.
+However, RPM, Distance/Odometer, Fuel Used, Vehicle Speed, Idle Status, Cruise Status, and other operational signals are available.
+Recommended Next Step:
+Develop and validate an FEI-Lite framework using currently available GeoTab telemetry data while preparing for future OEM data integration to enable Full FEI implementation.</t>
+  </si>
+  <si>
+    <t>- GeoTab provides several operational telemetry signals required for fleet analytics.
+- Critical Full FEI signals (Engine Load and Fuel Rate) were not observed in the DHL Hyundai pilot fleet.
+- Torque and Accelerator Pedal Position (APS) were also unavailable.
+- Available telemetry signals are sufficient to support development of an FEI-Lite framework.
+- Future OEM integration is recommended to enable Full FEI implementation.</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -45,13 +328,41 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -66,8 +377,39 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -402,6 +744,1100 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8401780C-9F4C-C740-9A03-556172335B4A}">
+  <dimension ref="A1:J72"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="4" max="4" width="18.33203125" customWidth="1"/>
+    <col min="5" max="5" width="21.83203125" customWidth="1"/>
+    <col min="6" max="6" width="15.83203125" customWidth="1"/>
+    <col min="7" max="7" width="15.5" customWidth="1"/>
+    <col min="8" max="8" width="15" customWidth="1"/>
+    <col min="9" max="9" width="37.1640625" customWidth="1"/>
+    <col min="10" max="10" width="62.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G2">
+        <v>12</v>
+      </c>
+      <c r="H2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G3">
+        <v>12</v>
+      </c>
+      <c r="H3" t="s">
+        <v>9</v>
+      </c>
+      <c r="I3" t="s">
+        <v>36</v>
+      </c>
+      <c r="J3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4">
+        <v>12</v>
+      </c>
+      <c r="H4" t="s">
+        <v>9</v>
+      </c>
+      <c r="I4" t="s">
+        <v>38</v>
+      </c>
+      <c r="J4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G5">
+        <v>12</v>
+      </c>
+      <c r="H5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I5" t="s">
+        <v>39</v>
+      </c>
+      <c r="J5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" t="s">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6" t="s">
+        <v>11</v>
+      </c>
+      <c r="I6" t="s">
+        <v>26</v>
+      </c>
+      <c r="J6" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" t="s">
+        <v>0</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7" t="s">
+        <v>11</v>
+      </c>
+      <c r="I7" t="s">
+        <v>26</v>
+      </c>
+      <c r="J7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>0</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8" t="s">
+        <v>11</v>
+      </c>
+      <c r="I8" t="s">
+        <v>42</v>
+      </c>
+      <c r="J8" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9" t="s">
+        <v>8</v>
+      </c>
+      <c r="F9" t="s">
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9" t="s">
+        <v>11</v>
+      </c>
+      <c r="I9" t="s">
+        <v>55</v>
+      </c>
+      <c r="J9" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" t="s">
+        <v>24</v>
+      </c>
+      <c r="D10" t="s">
+        <v>8</v>
+      </c>
+      <c r="E10" t="s">
+        <v>8</v>
+      </c>
+      <c r="F10" t="s">
+        <v>8</v>
+      </c>
+      <c r="G10">
+        <v>12</v>
+      </c>
+      <c r="H10" t="s">
+        <v>9</v>
+      </c>
+      <c r="I10" t="s">
+        <v>43</v>
+      </c>
+      <c r="J10" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11" t="s">
+        <v>0</v>
+      </c>
+      <c r="E11" t="s">
+        <v>8</v>
+      </c>
+      <c r="F11" t="s">
+        <v>8</v>
+      </c>
+      <c r="G11">
+        <v>12</v>
+      </c>
+      <c r="H11" t="s">
+        <v>9</v>
+      </c>
+      <c r="I11" t="s">
+        <v>45</v>
+      </c>
+      <c r="J11" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>47</v>
+      </c>
+      <c r="C12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" t="s">
+        <v>0</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>0</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12" t="s">
+        <v>11</v>
+      </c>
+      <c r="I12" t="s">
+        <v>19</v>
+      </c>
+      <c r="J12" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" t="s">
+        <v>16</v>
+      </c>
+      <c r="D13" t="s">
+        <v>0</v>
+      </c>
+      <c r="E13" t="s">
+        <v>8</v>
+      </c>
+      <c r="F13" t="s">
+        <v>8</v>
+      </c>
+      <c r="G13">
+        <v>12</v>
+      </c>
+      <c r="H13" t="s">
+        <v>9</v>
+      </c>
+      <c r="I13" t="s">
+        <v>49</v>
+      </c>
+      <c r="J13" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>51</v>
+      </c>
+      <c r="C14" t="s">
+        <v>16</v>
+      </c>
+      <c r="D14" t="s">
+        <v>0</v>
+      </c>
+      <c r="E14" t="s">
+        <v>8</v>
+      </c>
+      <c r="F14" t="s">
+        <v>8</v>
+      </c>
+      <c r="G14">
+        <v>12</v>
+      </c>
+      <c r="H14" t="s">
+        <v>9</v>
+      </c>
+      <c r="I14" t="s">
+        <v>52</v>
+      </c>
+      <c r="J14" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" t="s">
+        <v>16</v>
+      </c>
+      <c r="D15" t="s">
+        <v>0</v>
+      </c>
+      <c r="E15" t="s">
+        <v>8</v>
+      </c>
+      <c r="F15" t="s">
+        <v>8</v>
+      </c>
+      <c r="G15">
+        <v>12</v>
+      </c>
+      <c r="H15" t="s">
+        <v>9</v>
+      </c>
+      <c r="I15" t="s">
+        <v>54</v>
+      </c>
+      <c r="J15" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16" t="s">
+        <v>16</v>
+      </c>
+      <c r="D16" t="s">
+        <v>0</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>27</v>
+      </c>
+      <c r="G16" t="s">
+        <v>27</v>
+      </c>
+      <c r="H16" t="s">
+        <v>27</v>
+      </c>
+      <c r="I16" t="s">
+        <v>54</v>
+      </c>
+      <c r="J16" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>56</v>
+      </c>
+      <c r="C17" t="s">
+        <v>20</v>
+      </c>
+      <c r="D17" t="s">
+        <v>0</v>
+      </c>
+      <c r="E17" t="s">
+        <v>8</v>
+      </c>
+      <c r="F17" t="s">
+        <v>27</v>
+      </c>
+      <c r="G17" t="s">
+        <v>27</v>
+      </c>
+      <c r="H17" t="s">
+        <v>27</v>
+      </c>
+      <c r="I17" t="s">
+        <v>57</v>
+      </c>
+      <c r="J17" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>30</v>
+      </c>
+      <c r="C18" t="s">
+        <v>20</v>
+      </c>
+      <c r="D18" t="s">
+        <v>0</v>
+      </c>
+      <c r="E18" t="s">
+        <v>8</v>
+      </c>
+      <c r="F18" t="s">
+        <v>8</v>
+      </c>
+      <c r="G18">
+        <v>12</v>
+      </c>
+      <c r="H18" t="s">
+        <v>9</v>
+      </c>
+      <c r="I18" t="s">
+        <v>59</v>
+      </c>
+      <c r="J18" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>60</v>
+      </c>
+      <c r="C19" t="s">
+        <v>20</v>
+      </c>
+      <c r="D19" t="s">
+        <v>0</v>
+      </c>
+      <c r="E19" t="s">
+        <v>8</v>
+      </c>
+      <c r="F19" t="s">
+        <v>0</v>
+      </c>
+      <c r="G19">
+        <v>0</v>
+      </c>
+      <c r="H19" t="s">
+        <v>11</v>
+      </c>
+      <c r="I19" t="s">
+        <v>57</v>
+      </c>
+      <c r="J19" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>61</v>
+      </c>
+      <c r="C20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D20" t="s">
+        <v>0</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>0</v>
+      </c>
+      <c r="G20">
+        <v>0</v>
+      </c>
+      <c r="H20" t="s">
+        <v>11</v>
+      </c>
+      <c r="I20" t="s">
+        <v>57</v>
+      </c>
+      <c r="J20" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="24" x14ac:dyDescent="0.3">
+      <c r="A26" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A28" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B28" s="7"/>
+      <c r="C28" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="D28" s="4"/>
+      <c r="E28" s="4"/>
+      <c r="F28" s="4"/>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A29" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="B29" s="5"/>
+      <c r="C29" s="5">
+        <v>19</v>
+      </c>
+      <c r="D29" s="5"/>
+      <c r="E29" s="5"/>
+      <c r="F29" s="5"/>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A30" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="B30" s="5"/>
+      <c r="C30" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="D30" s="5"/>
+      <c r="E30" s="5"/>
+      <c r="F30" s="5"/>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A31" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B31" s="5"/>
+      <c r="C31" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="D31" s="6"/>
+      <c r="E31" s="6"/>
+      <c r="F31" s="6"/>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A32" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="B32" s="5"/>
+      <c r="C32" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="D32" s="5"/>
+      <c r="E32" s="5"/>
+      <c r="F32" s="5"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A33" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="B33" s="5"/>
+      <c r="C33" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D33" s="5"/>
+      <c r="E33" s="5"/>
+      <c r="F33" s="5"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A34" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="B34" s="5"/>
+      <c r="C34" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="D34" s="5"/>
+      <c r="E34" s="5"/>
+      <c r="F34" s="5"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A35" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B35" s="5"/>
+      <c r="C35" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D35" s="5"/>
+      <c r="E35" s="5"/>
+      <c r="F35" s="5"/>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A36" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="B36" s="5"/>
+      <c r="C36" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D36" s="5"/>
+      <c r="E36" s="5"/>
+      <c r="F36" s="5"/>
+    </row>
+    <row r="39" spans="1:6" ht="24" x14ac:dyDescent="0.3">
+      <c r="A39" s="3" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="11" t="s">
+        <v>85</v>
+      </c>
+      <c r="B40" s="8"/>
+      <c r="C40" s="8"/>
+      <c r="D40" s="8"/>
+      <c r="E40" s="8"/>
+      <c r="F40" s="8"/>
+    </row>
+    <row r="41" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="8"/>
+      <c r="B41" s="8"/>
+      <c r="C41" s="8"/>
+      <c r="D41" s="8"/>
+      <c r="E41" s="8"/>
+      <c r="F41" s="8"/>
+    </row>
+    <row r="42" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="8"/>
+      <c r="B42" s="8"/>
+      <c r="C42" s="8"/>
+      <c r="D42" s="8"/>
+      <c r="E42" s="8"/>
+      <c r="F42" s="8"/>
+    </row>
+    <row r="43" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="8"/>
+      <c r="B43" s="8"/>
+      <c r="C43" s="8"/>
+      <c r="D43" s="8"/>
+      <c r="E43" s="8"/>
+      <c r="F43" s="8"/>
+    </row>
+    <row r="44" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="8"/>
+      <c r="B44" s="8"/>
+      <c r="C44" s="8"/>
+      <c r="D44" s="8"/>
+      <c r="E44" s="8"/>
+      <c r="F44" s="8"/>
+    </row>
+    <row r="45" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="8"/>
+      <c r="B45" s="8"/>
+      <c r="C45" s="8"/>
+      <c r="D45" s="8"/>
+      <c r="E45" s="8"/>
+      <c r="F45" s="8"/>
+    </row>
+    <row r="46" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="8"/>
+      <c r="B46" s="8"/>
+      <c r="C46" s="8"/>
+      <c r="D46" s="8"/>
+      <c r="E46" s="8"/>
+      <c r="F46" s="8"/>
+    </row>
+    <row r="47" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="8"/>
+      <c r="B47" s="8"/>
+      <c r="C47" s="8"/>
+      <c r="D47" s="8"/>
+      <c r="E47" s="8"/>
+      <c r="F47" s="8"/>
+    </row>
+    <row r="48" spans="1:6" ht="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="8"/>
+      <c r="B48" s="8"/>
+      <c r="C48" s="8"/>
+      <c r="D48" s="8"/>
+      <c r="E48" s="8"/>
+      <c r="F48" s="8"/>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A49" s="8"/>
+      <c r="B49" s="8"/>
+      <c r="C49" s="8"/>
+      <c r="D49" s="8"/>
+      <c r="E49" s="8"/>
+      <c r="F49" s="8"/>
+    </row>
+    <row r="52" spans="1:7" ht="24" x14ac:dyDescent="0.3">
+      <c r="A52" s="3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A53" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="B53" s="9"/>
+      <c r="C53" s="9"/>
+      <c r="D53" s="9"/>
+      <c r="E53" s="9"/>
+      <c r="F53" s="9"/>
+      <c r="G53" s="9"/>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A54" s="9"/>
+      <c r="B54" s="9"/>
+      <c r="C54" s="9"/>
+      <c r="D54" s="9"/>
+      <c r="E54" s="9"/>
+      <c r="F54" s="9"/>
+      <c r="G54" s="9"/>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A55" s="9"/>
+      <c r="B55" s="9"/>
+      <c r="C55" s="9"/>
+      <c r="D55" s="9"/>
+      <c r="E55" s="9"/>
+      <c r="F55" s="9"/>
+      <c r="G55" s="9"/>
+    </row>
+    <row r="56" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A56" s="9"/>
+      <c r="B56" s="9"/>
+      <c r="C56" s="9"/>
+      <c r="D56" s="9"/>
+      <c r="E56" s="9"/>
+      <c r="F56" s="9"/>
+      <c r="G56" s="9"/>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A57" s="9"/>
+      <c r="B57" s="9"/>
+      <c r="C57" s="9"/>
+      <c r="D57" s="9"/>
+      <c r="E57" s="9"/>
+      <c r="F57" s="9"/>
+      <c r="G57" s="9"/>
+    </row>
+    <row r="58" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A58" s="9"/>
+      <c r="B58" s="9"/>
+      <c r="C58" s="9"/>
+      <c r="D58" s="9"/>
+      <c r="E58" s="9"/>
+      <c r="F58" s="9"/>
+      <c r="G58" s="9"/>
+    </row>
+    <row r="59" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A59" s="9"/>
+      <c r="B59" s="9"/>
+      <c r="C59" s="9"/>
+      <c r="D59" s="9"/>
+      <c r="E59" s="9"/>
+      <c r="F59" s="9"/>
+      <c r="G59" s="9"/>
+    </row>
+    <row r="60" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A60" s="9"/>
+      <c r="B60" s="9"/>
+      <c r="C60" s="9"/>
+      <c r="D60" s="9"/>
+      <c r="E60" s="9"/>
+      <c r="F60" s="9"/>
+      <c r="G60" s="9"/>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A61" s="9"/>
+      <c r="B61" s="9"/>
+      <c r="C61" s="9"/>
+      <c r="D61" s="9"/>
+      <c r="E61" s="9"/>
+      <c r="F61" s="9"/>
+      <c r="G61" s="9"/>
+    </row>
+    <row r="62" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A62" s="9"/>
+      <c r="B62" s="9"/>
+      <c r="C62" s="9"/>
+      <c r="D62" s="9"/>
+      <c r="E62" s="9"/>
+      <c r="F62" s="9"/>
+      <c r="G62" s="9"/>
+    </row>
+    <row r="63" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A63" s="9"/>
+      <c r="B63" s="9"/>
+      <c r="C63" s="9"/>
+      <c r="D63" s="9"/>
+      <c r="E63" s="9"/>
+      <c r="F63" s="9"/>
+      <c r="G63" s="9"/>
+    </row>
+    <row r="64" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A64" s="9"/>
+      <c r="B64" s="9"/>
+      <c r="C64" s="9"/>
+      <c r="D64" s="9"/>
+      <c r="E64" s="9"/>
+      <c r="F64" s="9"/>
+      <c r="G64" s="9"/>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A65" s="9"/>
+      <c r="B65" s="9"/>
+      <c r="C65" s="9"/>
+      <c r="D65" s="9"/>
+      <c r="E65" s="9"/>
+      <c r="F65" s="9"/>
+      <c r="G65" s="9"/>
+    </row>
+    <row r="66" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A66" s="9"/>
+      <c r="B66" s="9"/>
+      <c r="C66" s="9"/>
+      <c r="D66" s="9"/>
+      <c r="E66" s="9"/>
+      <c r="F66" s="9"/>
+      <c r="G66" s="9"/>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A67" s="9"/>
+      <c r="B67" s="9"/>
+      <c r="C67" s="9"/>
+      <c r="D67" s="9"/>
+      <c r="E67" s="9"/>
+      <c r="F67" s="9"/>
+      <c r="G67" s="9"/>
+    </row>
+    <row r="68" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A68" s="9"/>
+      <c r="B68" s="9"/>
+      <c r="C68" s="9"/>
+      <c r="D68" s="9"/>
+      <c r="E68" s="9"/>
+      <c r="F68" s="9"/>
+      <c r="G68" s="9"/>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A69" s="9"/>
+      <c r="B69" s="9"/>
+      <c r="C69" s="9"/>
+      <c r="D69" s="9"/>
+      <c r="E69" s="9"/>
+      <c r="F69" s="9"/>
+      <c r="G69" s="9"/>
+    </row>
+    <row r="70" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A70" s="9"/>
+      <c r="B70" s="9"/>
+      <c r="C70" s="9"/>
+      <c r="D70" s="9"/>
+      <c r="E70" s="9"/>
+      <c r="F70" s="9"/>
+      <c r="G70" s="9"/>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A71" s="9"/>
+      <c r="B71" s="9"/>
+      <c r="C71" s="9"/>
+      <c r="D71" s="9"/>
+      <c r="E71" s="9"/>
+      <c r="F71" s="9"/>
+      <c r="G71" s="9"/>
+    </row>
+    <row r="72" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A72" s="9"/>
+      <c r="B72" s="9"/>
+      <c r="C72" s="9"/>
+      <c r="D72" s="9"/>
+      <c r="E72" s="9"/>
+      <c r="F72" s="9"/>
+      <c r="G72" s="9"/>
+    </row>
+  </sheetData>
+  <mergeCells count="19">
+    <mergeCell ref="A40:F49"/>
+    <mergeCell ref="A53:G72"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="C34:F34"/>
+    <mergeCell ref="C29:F29"/>
+    <mergeCell ref="C28:F28"/>
+    <mergeCell ref="C35:F35"/>
+    <mergeCell ref="C36:F36"/>
+    <mergeCell ref="C32:F32"/>
+    <mergeCell ref="C30:F30"/>
+    <mergeCell ref="C33:F33"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A30:B30"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B8526C6-7212-EE4B-BB25-602DDD881251}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9647CE43-ED5F-CF49-B719-99CBC527DB3E}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CC2A96B-595B-E747-BF11-6EEB10631C05}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B924726-B2AB-6640-9A1C-88ACA9E2EEDE}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData/>

</xml_diff>

<commit_message>
Add FEI-Lite methodology and data dictionary
</commit_message>
<xml_diff>
--- a/docs/signal_availability_matrix.xlsx
+++ b/docs/signal_availability_matrix.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/haneuljang/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/haneuljang/Desktop/fleet-telemetry-analytics/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F253B4F2-62A2-5248-AE1B-DB13A59C31FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBA30427-3E01-6D48-8AA7-AE02814357FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="21360" activeTab="3" xr2:uid="{29318AA6-4BD7-6244-B5A3-8C80AA045784}"/>
+    <workbookView xWindow="2480" yWindow="22380" windowWidth="34200" windowHeight="21360" activeTab="4" xr2:uid="{29318AA6-4BD7-6244-B5A3-8C80AA045784}"/>
   </bookViews>
   <sheets>
     <sheet name="FEI Signal Validation" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="Signal Gap Analysis" sheetId="4" r:id="rId4"/>
     <sheet name="OEM Limitation Summary" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="613" uniqueCount="216">
   <si>
     <t>No</t>
   </si>
@@ -295,7 +295,128 @@
     <t>Required FEI Signals Evaluated | 19</t>
   </si>
   <si>
-    <t>Validation Result
+    <t>- GeoTab provides several operational telemetry signals required for fleet analytics.
+- Critical Full FEI signals (Engine Load and Fuel Rate) were not observed in the DHL Hyundai pilot fleet.
+- Torque and Accelerator Pedal Position (APS) were also unavailable.
+- Available telemetry signals are sufficient to support development of an FEI-Lite framework.
+- Future OEM integration is recommended to enable Full FEI implementation.</t>
+  </si>
+  <si>
+    <t>Required for Full DSI</t>
+  </si>
+  <si>
+    <t>Supports regeneration analysis</t>
+  </si>
+  <si>
+    <t>DPF Differential Pressure</t>
+  </si>
+  <si>
+    <t>DPF Intake Temperature</t>
+  </si>
+  <si>
+    <t>DPF Outlet Temperature</t>
+  </si>
+  <si>
+    <t>DPF Soot Load</t>
+  </si>
+  <si>
+    <t>Regeneration Status</t>
+  </si>
+  <si>
+    <t>Regeneration Count</t>
+  </si>
+  <si>
+    <t>Fuel Used</t>
+  </si>
+  <si>
+    <t>Supports operating condition analysis</t>
+  </si>
+  <si>
+    <t>DSI Validation Summary</t>
+  </si>
+  <si>
+    <t>Required DSI Signals Evaluated</t>
+  </si>
+  <si>
+    <t>Full DSI Feasible</t>
+  </si>
+  <si>
+    <t>DSI-Lite Feasible</t>
+  </si>
+  <si>
+    <t>DHL Pilot Data 
+Available</t>
+  </si>
+  <si>
+    <t>Vehicle Count
+ With Data</t>
+  </si>
+  <si>
+    <t>Not observed in current validation dataset</t>
+  </si>
+  <si>
+    <t>Critical DPF health indicator</t>
+  </si>
+  <si>
+    <t>Observed on vehicle 93나2374 only</t>
+  </si>
+  <si>
+    <t>Supports regeneration monitoring</t>
+  </si>
+  <si>
+    <t>Supports regeneration validation</t>
+  </si>
+  <si>
+    <t>Required for DPF loading assessment</t>
+  </si>
+  <si>
+    <t>Not observed in pilot fleet</t>
+  </si>
+  <si>
+    <t>Required for regeneration tracking</t>
+  </si>
+  <si>
+    <t>Required for regeneration frequency analysis</t>
+  </si>
+  <si>
+    <t>Supports fuel impact calculations</t>
+  </si>
+  <si>
+    <t>Vehicle Speed available</t>
+  </si>
+  <si>
+    <t>Vehicle Speed Available</t>
+  </si>
+  <si>
+    <t>DPF Differential Pressure, DPF Intake Temperature, DPF Outlet Temperature</t>
+  </si>
+  <si>
+    <t>Engine RPM, Fuel Used, Vehicle Speed</t>
+  </si>
+  <si>
+    <t>DPF Soot Load, Regeneration Status, Regeneration Count</t>
+  </si>
+  <si>
+    <t>Limited Availability Signals</t>
+  </si>
+  <si>
+    <t>DPF Pressure &amp; Temperature Signals</t>
+  </si>
+  <si>
+    <t>Partial DSI Feasible</t>
+  </si>
+  <si>
+    <t>• GeoTab is capable of collecting DPF-related diagnostics.
+• Critical DPF telemetry signals including DPF Differential Pressure, DPF Intake Temperature, and DPF Outlet Temperature were observed within the DHL pilot fleet.
+• However, these signals were only available on a limited subset of vehicles and were not consistently available fleet-wide.
+• DPF Soot Load, Regeneration Status, and Regeneration Count were not observed.
+• Full DSI implementation is not currently feasible, but a DSI-Lite framework can be developed using available DPF diagnostics.</t>
+  </si>
+  <si>
+    <t>Validation Result</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validation Result
 The DHL Hyundai pilot fleet does not currently provide the critical telemetry signals required for Full FEI implementation.
 Missing Critical Signals:
 - Engine Load
@@ -305,22 +426,333 @@
 - Accelerator Pedal Position (APS)
 Therefore, Full FEI implementation is not currently feasible.
 However, RPM, Distance/Odometer, Fuel Used, Vehicle Speed, Idle Status, Cruise Status, and other operational signals are available.
-Recommended Next Step:
-Develop and validate an FEI-Lite framework using currently available GeoTab telemetry data while preparing for future OEM data integration to enable Full FEI implementation.</t>
-  </si>
-  <si>
-    <t>- GeoTab provides several operational telemetry signals required for fleet analytics.
-- Critical Full FEI signals (Engine Load and Fuel Rate) were not observed in the DHL Hyundai pilot fleet.
-- Torque and Accelerator Pedal Position (APS) were also unavailable.
-- Available telemetry signals are sufficient to support development of an FEI-Lite framework.
-- Future OEM integration is recommended to enable Full FEI implementation.</t>
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validation Result
+The DHL Hyundai pilot fleet provides partial access to DPF-related telemetry signals required for Diesel Sustainability Index (DSI) implementation.
+Available DSI Signals:
+- DPF Differential Pressure
+- DPF Intake Temperature
+- DPF Outlet Temperature
+- Engine RPM
+- Fuel Used
+- Vehicle Speed
+Missing Critical Signals:
+- DPF Soot Load
+- Regeneration Status
+- Regeneration Count
+Because critical DSI signals are only available on a limited number of vehicles, fleet-wide Full DSI implementation is not currently feasible.
+However, DSI-Lite development is feasible and can be used to evaluate DPF thermal behavior and regeneration-related operating conditions.
+</t>
+  </si>
+  <si>
+    <t>Required for Full VEI</t>
+  </si>
+  <si>
+    <t>Supports emissions normalization</t>
+  </si>
+  <si>
+    <t>Supports fuel-related emission estimation</t>
+  </si>
+  <si>
+    <t>NOx Concentration</t>
+  </si>
+  <si>
+    <t>Core VEI parameter</t>
+  </si>
+  <si>
+    <t>Not observed in DHL pilot fleet</t>
+  </si>
+  <si>
+    <t>SCR Efficiency</t>
+  </si>
+  <si>
+    <t>Required for aftertreatment performance analysis</t>
+  </si>
+  <si>
+    <t>DPF Emission Data</t>
+  </si>
+  <si>
+    <t>Required for particulate emission assessment</t>
+  </si>
+  <si>
+    <t>Improves emission modeling</t>
+  </si>
+  <si>
+    <t>Engine Torque</t>
+  </si>
+  <si>
+    <t>Improves engine work estimation</t>
+  </si>
+  <si>
+    <t>Engine Coolant Temperature</t>
+  </si>
+  <si>
+    <t>Engine Oil Temperature</t>
+  </si>
+  <si>
+    <t>DHL Pilo
+ Data Available</t>
+  </si>
+  <si>
+    <t>Vehicle Count 
+With Data</t>
+  </si>
+  <si>
+    <t>VEI Validation Summary</t>
+  </si>
+  <si>
+    <t>Required VEI Signals Evaluated</t>
+  </si>
+  <si>
+    <t>RPM, Vehicle Speed, Fuel Used</t>
+  </si>
+  <si>
+    <t>Coolant Temperature, Oil Temperature</t>
+  </si>
+  <si>
+    <t>NOx Concentration, SCR Efficiency, DPF Emission Data</t>
+  </si>
+  <si>
+    <t>Engine Load, Engine Torque</t>
+  </si>
+  <si>
+    <t>Full VEI Feasible</t>
+  </si>
+  <si>
+    <t>VEI-Lite Feasible</t>
+  </si>
+  <si>
+    <t>Future OEM Integration Required</t>
+  </si>
+  <si>
+    <t>• GeoTab provides several operational signals that may support emission-related analytics.
+• Critical emission diagnostics including NOx Concentration, SCR Efficiency, and DPF Emission data were not observed in the DHL Hyundai pilot fleet.
+• Engine Load and Engine Torque were also unavailable.
+• Available telemetry signals are insufficient to support development of a scientifically valid VEI framework.
+• Additional OEM-level emission diagnostics are required before VEI implementation can be considered.</t>
+  </si>
+  <si>
+    <t>Validation Result
+The DHL Hyundai pilot fleet does not currently provide the critical emission-related signals required for Vehicle Emission Index (VEI) implementation.
+Available Signals:
+- Engine RPM
+- Vehicle Speed
+- Fuel Used
+- Engine Coolant Temperature
+- Engine Oil Temperature
+Missing Critical Signals:
+- NOx Concentration
+- SCR Efficiency
+- DPF Emission Data
+Missing Additional Signals:
+- Engine Load
+- Engine Torque
+Therefore, Full VEI implementation is not currently feasible.
+Unlike FEI-Lite and DSI-Lite, the available telemetry data are insufficient to support a reliable VEI-Lite framework.</t>
+  </si>
+  <si>
+    <t>Framework</t>
+  </si>
+  <si>
+    <t>Required Signal</t>
+  </si>
+  <si>
+    <t>Current Status</t>
+  </si>
+  <si>
+    <t>Impact</t>
+  </si>
+  <si>
+    <t>Recommended Action</t>
+  </si>
+  <si>
+    <t>FEI</t>
+  </si>
+  <si>
+    <t>Missing</t>
+  </si>
+  <si>
+    <t>Full FEI calculation not possible</t>
+  </si>
+  <si>
+    <t>Request OEM ECU data</t>
+  </si>
+  <si>
+    <t>Fuel efficiency normalization limited</t>
+  </si>
+  <si>
+    <t>Engine work estimation unavailable</t>
+  </si>
+  <si>
+    <t>Accelerator Pedal Position</t>
+  </si>
+  <si>
+    <t>Driver demand analysis limited</t>
+  </si>
+  <si>
+    <t>DSI</t>
+  </si>
+  <si>
+    <t>DPF loading assessment unavailable</t>
+  </si>
+  <si>
+    <t>Request OEM DPF data</t>
+  </si>
+  <si>
+    <t>Regeneration monitoring unavailable</t>
+  </si>
+  <si>
+    <t>Regeneration frequency analysis unavailable</t>
+  </si>
+  <si>
+    <t>VEI</t>
+  </si>
+  <si>
+    <t>Emission estimation not possible</t>
+  </si>
+  <si>
+    <t>Request OEM emissions data</t>
+  </si>
+  <si>
+    <t>Aftertreatment performance unavailable</t>
+  </si>
+  <si>
+    <t>Emission scoring unavailable</t>
+  </si>
+  <si>
+    <t>Signal Gap Analysis Summary</t>
+  </si>
+  <si>
+    <t>Total Signals Evaluated</t>
+  </si>
+  <si>
+    <t>Available Signals</t>
+  </si>
+  <si>
+    <t>Missing Signals</t>
+  </si>
+  <si>
+    <t>Partial Signals</t>
+  </si>
+  <si>
+    <t>• Several high-value operational signals were successfully collected through GeoTab.</t>
+  </si>
+  <si>
+    <t>• Critical FEI signals including Engine Load, Fuel Rate, and Torque were not available.</t>
+  </si>
+  <si>
+    <t>• DPF-related diagnostics were partially available but not fleet-wide.</t>
+  </si>
+  <si>
+    <t>• Core emissions diagnostics including NOx and SCR efficiency were unavailable.</t>
+  </si>
+  <si>
+    <t>• OEM-level access is required to enable Full FEI, DSI, and VEI implementation.</t>
+  </si>
+  <si>
+    <t>GeoTab Platform Support</t>
+  </si>
+  <si>
+    <t>DHL Fleet Availability</t>
+  </si>
+  <si>
+    <t>Limitation Type</t>
+  </si>
+  <si>
+    <t>OEM Limitation</t>
+  </si>
+  <si>
+    <t>Full FEI unavailable</t>
+  </si>
+  <si>
+    <t>Possible</t>
+  </si>
+  <si>
+    <t>Reduced model accuracy</t>
+  </si>
+  <si>
+    <t>Limited driver behavior analysis</t>
+  </si>
+  <si>
+    <t>Vehicle Configuration Limitation</t>
+  </si>
+  <si>
+    <t>Partial DSI only</t>
+  </si>
+  <si>
+    <t>Full DSI unavailable</t>
+  </si>
+  <si>
+    <t>Full VEI unavailable</t>
+  </si>
+  <si>
+    <t>OEM Limitation Summary</t>
+  </si>
+  <si>
+    <t>GeoTab Platform Capability</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>DHL Fleet Signal Availability</t>
+  </si>
+  <si>
+    <t>Limited</t>
+  </si>
+  <si>
+    <t>FEI Limitation Source</t>
+  </si>
+  <si>
+    <t>Missing OEM engine diagnostics</t>
+  </si>
+  <si>
+    <t>DSI Limitation Source</t>
+  </si>
+  <si>
+    <t>Missing OEM DPF diagnostics</t>
+  </si>
+  <si>
+    <t>VEI Limitation Source</t>
+  </si>
+  <si>
+    <t>Missing OEM emissions diagnostics</t>
+  </si>
+  <si>
+    <t>Additional OEM Integration Required</t>
+  </si>
+  <si>
+    <t>The GeoTab platform is technically capable of supporting advanced</t>
+  </si>
+  <si>
+    <t>fleet analytics, including fuel-efficiency, DPF-health, and</t>
+  </si>
+  <si>
+    <t>emissions-related monitoring.</t>
+  </si>
+  <si>
+    <t>However, several critical diagnostics required for Full FEI,</t>
+  </si>
+  <si>
+    <t>DSI, and VEI implementation were not available within the</t>
+  </si>
+  <si>
+    <t>current DHL Hyundai pilot fleet.</t>
+  </si>
+  <si>
+    <t>The primary limitation is not the GeoTab platform itself,</t>
+  </si>
+  <si>
+    <t>but the availability of OEM-specific ECU diagnostics.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -350,8 +782,29 @@
       <name val="Arial Unicode MS"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="24"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="24"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow (Body)"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -361,6 +814,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -377,38 +836,54 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" shrinkToFit="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -757,34 +1232,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="13" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1397,394 +1872,404 @@
       </c>
     </row>
     <row r="26" spans="1:10" ht="24" x14ac:dyDescent="0.3">
-      <c r="A26" s="3" t="s">
+      <c r="A26" s="1" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A28" s="7" t="s">
+      <c r="A28" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="B28" s="7"/>
-      <c r="C28" s="4" t="s">
+      <c r="B28" s="9"/>
+      <c r="C28" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="D28" s="4"/>
-      <c r="E28" s="4"/>
-      <c r="F28" s="4"/>
+      <c r="D28" s="8"/>
+      <c r="E28" s="8"/>
+      <c r="F28" s="8"/>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A29" s="5" t="s">
+      <c r="A29" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="B29" s="5"/>
-      <c r="C29" s="5">
+      <c r="B29" s="7"/>
+      <c r="C29" s="7">
         <v>19</v>
       </c>
-      <c r="D29" s="5"/>
-      <c r="E29" s="5"/>
-      <c r="F29" s="5"/>
+      <c r="D29" s="7"/>
+      <c r="E29" s="7"/>
+      <c r="F29" s="7"/>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A30" s="5" t="s">
+      <c r="A30" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="B30" s="5"/>
-      <c r="C30" s="5" t="s">
+      <c r="B30" s="7"/>
+      <c r="C30" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="D30" s="5"/>
-      <c r="E30" s="5"/>
-      <c r="F30" s="5"/>
+      <c r="D30" s="7"/>
+      <c r="E30" s="7"/>
+      <c r="F30" s="7"/>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A31" s="5" t="s">
+      <c r="A31" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="B31" s="5"/>
-      <c r="C31" s="6" t="s">
+      <c r="B31" s="7"/>
+      <c r="C31" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="D31" s="6"/>
-      <c r="E31" s="6"/>
-      <c r="F31" s="6"/>
+      <c r="D31" s="2"/>
+      <c r="E31" s="2"/>
+      <c r="F31" s="2"/>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A32" s="5" t="s">
+      <c r="A32" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="B32" s="5"/>
-      <c r="C32" s="5" t="s">
+      <c r="B32" s="7"/>
+      <c r="C32" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="D32" s="5"/>
-      <c r="E32" s="5"/>
-      <c r="F32" s="5"/>
+      <c r="D32" s="7"/>
+      <c r="E32" s="7"/>
+      <c r="F32" s="7"/>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A33" s="5" t="s">
+      <c r="A33" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="B33" s="5"/>
-      <c r="C33" s="5" t="s">
+      <c r="B33" s="7"/>
+      <c r="C33" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="D33" s="5"/>
-      <c r="E33" s="5"/>
-      <c r="F33" s="5"/>
+      <c r="D33" s="7"/>
+      <c r="E33" s="7"/>
+      <c r="F33" s="7"/>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A34" s="5" t="s">
+      <c r="A34" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="B34" s="5"/>
-      <c r="C34" s="5" t="s">
+      <c r="B34" s="7"/>
+      <c r="C34" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="D34" s="5"/>
-      <c r="E34" s="5"/>
-      <c r="F34" s="5"/>
+      <c r="D34" s="7"/>
+      <c r="E34" s="7"/>
+      <c r="F34" s="7"/>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A35" s="5" t="s">
+      <c r="A35" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="B35" s="5"/>
-      <c r="C35" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D35" s="5"/>
-      <c r="E35" s="5"/>
-      <c r="F35" s="5"/>
+      <c r="B35" s="7"/>
+      <c r="C35" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="D35" s="7"/>
+      <c r="E35" s="7"/>
+      <c r="F35" s="7"/>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A36" s="5" t="s">
+      <c r="A36" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="B36" s="5"/>
-      <c r="C36" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D36" s="5"/>
-      <c r="E36" s="5"/>
-      <c r="F36" s="5"/>
+      <c r="B36" s="7"/>
+      <c r="C36" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D36" s="7"/>
+      <c r="E36" s="7"/>
+      <c r="F36" s="7"/>
     </row>
     <row r="39" spans="1:6" ht="24" x14ac:dyDescent="0.3">
-      <c r="A39" s="3" t="s">
+      <c r="A39" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="B40" s="8"/>
-      <c r="C40" s="8"/>
-      <c r="D40" s="8"/>
-      <c r="E40" s="8"/>
-      <c r="F40" s="8"/>
+      <c r="A40" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B40" s="4"/>
+      <c r="C40" s="4"/>
+      <c r="D40" s="4"/>
+      <c r="E40" s="4"/>
+      <c r="F40" s="4"/>
     </row>
     <row r="41" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="8"/>
-      <c r="B41" s="8"/>
-      <c r="C41" s="8"/>
-      <c r="D41" s="8"/>
-      <c r="E41" s="8"/>
-      <c r="F41" s="8"/>
+      <c r="A41" s="4"/>
+      <c r="B41" s="4"/>
+      <c r="C41" s="4"/>
+      <c r="D41" s="4"/>
+      <c r="E41" s="4"/>
+      <c r="F41" s="4"/>
     </row>
     <row r="42" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="8"/>
-      <c r="B42" s="8"/>
-      <c r="C42" s="8"/>
-      <c r="D42" s="8"/>
-      <c r="E42" s="8"/>
-      <c r="F42" s="8"/>
+      <c r="A42" s="4"/>
+      <c r="B42" s="4"/>
+      <c r="C42" s="4"/>
+      <c r="D42" s="4"/>
+      <c r="E42" s="4"/>
+      <c r="F42" s="4"/>
     </row>
     <row r="43" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="8"/>
-      <c r="B43" s="8"/>
-      <c r="C43" s="8"/>
-      <c r="D43" s="8"/>
-      <c r="E43" s="8"/>
-      <c r="F43" s="8"/>
+      <c r="A43" s="4"/>
+      <c r="B43" s="4"/>
+      <c r="C43" s="4"/>
+      <c r="D43" s="4"/>
+      <c r="E43" s="4"/>
+      <c r="F43" s="4"/>
     </row>
     <row r="44" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="8"/>
-      <c r="B44" s="8"/>
-      <c r="C44" s="8"/>
-      <c r="D44" s="8"/>
-      <c r="E44" s="8"/>
-      <c r="F44" s="8"/>
+      <c r="A44" s="4"/>
+      <c r="B44" s="4"/>
+      <c r="C44" s="4"/>
+      <c r="D44" s="4"/>
+      <c r="E44" s="4"/>
+      <c r="F44" s="4"/>
     </row>
     <row r="45" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="8"/>
-      <c r="B45" s="8"/>
-      <c r="C45" s="8"/>
-      <c r="D45" s="8"/>
-      <c r="E45" s="8"/>
-      <c r="F45" s="8"/>
+      <c r="A45" s="4"/>
+      <c r="B45" s="4"/>
+      <c r="C45" s="4"/>
+      <c r="D45" s="4"/>
+      <c r="E45" s="4"/>
+      <c r="F45" s="4"/>
     </row>
     <row r="46" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="8"/>
-      <c r="B46" s="8"/>
-      <c r="C46" s="8"/>
-      <c r="D46" s="8"/>
-      <c r="E46" s="8"/>
-      <c r="F46" s="8"/>
+      <c r="A46" s="4"/>
+      <c r="B46" s="4"/>
+      <c r="C46" s="4"/>
+      <c r="D46" s="4"/>
+      <c r="E46" s="4"/>
+      <c r="F46" s="4"/>
     </row>
     <row r="47" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="8"/>
-      <c r="B47" s="8"/>
-      <c r="C47" s="8"/>
-      <c r="D47" s="8"/>
-      <c r="E47" s="8"/>
-      <c r="F47" s="8"/>
+      <c r="A47" s="4"/>
+      <c r="B47" s="4"/>
+      <c r="C47" s="4"/>
+      <c r="D47" s="4"/>
+      <c r="E47" s="4"/>
+      <c r="F47" s="4"/>
     </row>
     <row r="48" spans="1:6" ht="1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="8"/>
-      <c r="B48" s="8"/>
-      <c r="C48" s="8"/>
-      <c r="D48" s="8"/>
-      <c r="E48" s="8"/>
-      <c r="F48" s="8"/>
+      <c r="A48" s="4"/>
+      <c r="B48" s="4"/>
+      <c r="C48" s="4"/>
+      <c r="D48" s="4"/>
+      <c r="E48" s="4"/>
+      <c r="F48" s="4"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A49" s="8"/>
-      <c r="B49" s="8"/>
-      <c r="C49" s="8"/>
-      <c r="D49" s="8"/>
-      <c r="E49" s="8"/>
-      <c r="F49" s="8"/>
+      <c r="A49" s="4"/>
+      <c r="B49" s="4"/>
+      <c r="C49" s="4"/>
+      <c r="D49" s="4"/>
+      <c r="E49" s="4"/>
+      <c r="F49" s="4"/>
     </row>
     <row r="52" spans="1:7" ht="24" x14ac:dyDescent="0.3">
-      <c r="A52" s="3" t="s">
+      <c r="A52" s="1" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A53" s="10" t="s">
-        <v>84</v>
-      </c>
-      <c r="B53" s="9"/>
-      <c r="C53" s="9"/>
-      <c r="D53" s="9"/>
-      <c r="E53" s="9"/>
-      <c r="F53" s="9"/>
-      <c r="G53" s="9"/>
+      <c r="A53" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="B53" s="6"/>
+      <c r="C53" s="6"/>
+      <c r="D53" s="6"/>
+      <c r="E53" s="6"/>
+      <c r="F53" s="6"/>
+      <c r="G53" s="6"/>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A54" s="9"/>
-      <c r="B54" s="9"/>
-      <c r="C54" s="9"/>
-      <c r="D54" s="9"/>
-      <c r="E54" s="9"/>
-      <c r="F54" s="9"/>
-      <c r="G54" s="9"/>
+      <c r="A54" s="6"/>
+      <c r="B54" s="6"/>
+      <c r="C54" s="6"/>
+      <c r="D54" s="6"/>
+      <c r="E54" s="6"/>
+      <c r="F54" s="6"/>
+      <c r="G54" s="6"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A55" s="9"/>
-      <c r="B55" s="9"/>
-      <c r="C55" s="9"/>
-      <c r="D55" s="9"/>
-      <c r="E55" s="9"/>
-      <c r="F55" s="9"/>
-      <c r="G55" s="9"/>
+      <c r="A55" s="6"/>
+      <c r="B55" s="6"/>
+      <c r="C55" s="6"/>
+      <c r="D55" s="6"/>
+      <c r="E55" s="6"/>
+      <c r="F55" s="6"/>
+      <c r="G55" s="6"/>
     </row>
     <row r="56" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="9"/>
-      <c r="B56" s="9"/>
-      <c r="C56" s="9"/>
-      <c r="D56" s="9"/>
-      <c r="E56" s="9"/>
-      <c r="F56" s="9"/>
-      <c r="G56" s="9"/>
+      <c r="A56" s="6"/>
+      <c r="B56" s="6"/>
+      <c r="C56" s="6"/>
+      <c r="D56" s="6"/>
+      <c r="E56" s="6"/>
+      <c r="F56" s="6"/>
+      <c r="G56" s="6"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A57" s="9"/>
-      <c r="B57" s="9"/>
-      <c r="C57" s="9"/>
-      <c r="D57" s="9"/>
-      <c r="E57" s="9"/>
-      <c r="F57" s="9"/>
-      <c r="G57" s="9"/>
+      <c r="A57" s="6"/>
+      <c r="B57" s="6"/>
+      <c r="C57" s="6"/>
+      <c r="D57" s="6"/>
+      <c r="E57" s="6"/>
+      <c r="F57" s="6"/>
+      <c r="G57" s="6"/>
     </row>
     <row r="58" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="9"/>
-      <c r="B58" s="9"/>
-      <c r="C58" s="9"/>
-      <c r="D58" s="9"/>
-      <c r="E58" s="9"/>
-      <c r="F58" s="9"/>
-      <c r="G58" s="9"/>
+      <c r="A58" s="6"/>
+      <c r="B58" s="6"/>
+      <c r="C58" s="6"/>
+      <c r="D58" s="6"/>
+      <c r="E58" s="6"/>
+      <c r="F58" s="6"/>
+      <c r="G58" s="6"/>
     </row>
     <row r="59" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="9"/>
-      <c r="B59" s="9"/>
-      <c r="C59" s="9"/>
-      <c r="D59" s="9"/>
-      <c r="E59" s="9"/>
-      <c r="F59" s="9"/>
-      <c r="G59" s="9"/>
+      <c r="A59" s="6"/>
+      <c r="B59" s="6"/>
+      <c r="C59" s="6"/>
+      <c r="D59" s="6"/>
+      <c r="E59" s="6"/>
+      <c r="F59" s="6"/>
+      <c r="G59" s="6"/>
     </row>
     <row r="60" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="9"/>
-      <c r="B60" s="9"/>
-      <c r="C60" s="9"/>
-      <c r="D60" s="9"/>
-      <c r="E60" s="9"/>
-      <c r="F60" s="9"/>
-      <c r="G60" s="9"/>
+      <c r="A60" s="6"/>
+      <c r="B60" s="6"/>
+      <c r="C60" s="6"/>
+      <c r="D60" s="6"/>
+      <c r="E60" s="6"/>
+      <c r="F60" s="6"/>
+      <c r="G60" s="6"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A61" s="9"/>
-      <c r="B61" s="9"/>
-      <c r="C61" s="9"/>
-      <c r="D61" s="9"/>
-      <c r="E61" s="9"/>
-      <c r="F61" s="9"/>
-      <c r="G61" s="9"/>
+      <c r="A61" s="6"/>
+      <c r="B61" s="6"/>
+      <c r="C61" s="6"/>
+      <c r="D61" s="6"/>
+      <c r="E61" s="6"/>
+      <c r="F61" s="6"/>
+      <c r="G61" s="6"/>
     </row>
     <row r="62" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="9"/>
-      <c r="B62" s="9"/>
-      <c r="C62" s="9"/>
-      <c r="D62" s="9"/>
-      <c r="E62" s="9"/>
-      <c r="F62" s="9"/>
-      <c r="G62" s="9"/>
+      <c r="A62" s="6"/>
+      <c r="B62" s="6"/>
+      <c r="C62" s="6"/>
+      <c r="D62" s="6"/>
+      <c r="E62" s="6"/>
+      <c r="F62" s="6"/>
+      <c r="G62" s="6"/>
     </row>
     <row r="63" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A63" s="9"/>
-      <c r="B63" s="9"/>
-      <c r="C63" s="9"/>
-      <c r="D63" s="9"/>
-      <c r="E63" s="9"/>
-      <c r="F63" s="9"/>
-      <c r="G63" s="9"/>
+      <c r="A63" s="6"/>
+      <c r="B63" s="6"/>
+      <c r="C63" s="6"/>
+      <c r="D63" s="6"/>
+      <c r="E63" s="6"/>
+      <c r="F63" s="6"/>
+      <c r="G63" s="6"/>
     </row>
     <row r="64" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A64" s="9"/>
-      <c r="B64" s="9"/>
-      <c r="C64" s="9"/>
-      <c r="D64" s="9"/>
-      <c r="E64" s="9"/>
-      <c r="F64" s="9"/>
-      <c r="G64" s="9"/>
+      <c r="A64" s="6"/>
+      <c r="B64" s="6"/>
+      <c r="C64" s="6"/>
+      <c r="D64" s="6"/>
+      <c r="E64" s="6"/>
+      <c r="F64" s="6"/>
+      <c r="G64" s="6"/>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A65" s="9"/>
-      <c r="B65" s="9"/>
-      <c r="C65" s="9"/>
-      <c r="D65" s="9"/>
-      <c r="E65" s="9"/>
-      <c r="F65" s="9"/>
-      <c r="G65" s="9"/>
+      <c r="A65" s="6"/>
+      <c r="B65" s="6"/>
+      <c r="C65" s="6"/>
+      <c r="D65" s="6"/>
+      <c r="E65" s="6"/>
+      <c r="F65" s="6"/>
+      <c r="G65" s="6"/>
     </row>
     <row r="66" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A66" s="9"/>
-      <c r="B66" s="9"/>
-      <c r="C66" s="9"/>
-      <c r="D66" s="9"/>
-      <c r="E66" s="9"/>
-      <c r="F66" s="9"/>
-      <c r="G66" s="9"/>
+      <c r="A66" s="6"/>
+      <c r="B66" s="6"/>
+      <c r="C66" s="6"/>
+      <c r="D66" s="6"/>
+      <c r="E66" s="6"/>
+      <c r="F66" s="6"/>
+      <c r="G66" s="6"/>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A67" s="9"/>
-      <c r="B67" s="9"/>
-      <c r="C67" s="9"/>
-      <c r="D67" s="9"/>
-      <c r="E67" s="9"/>
-      <c r="F67" s="9"/>
-      <c r="G67" s="9"/>
+      <c r="A67" s="6"/>
+      <c r="B67" s="6"/>
+      <c r="C67" s="6"/>
+      <c r="D67" s="6"/>
+      <c r="E67" s="6"/>
+      <c r="F67" s="6"/>
+      <c r="G67" s="6"/>
     </row>
     <row r="68" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A68" s="9"/>
-      <c r="B68" s="9"/>
-      <c r="C68" s="9"/>
-      <c r="D68" s="9"/>
-      <c r="E68" s="9"/>
-      <c r="F68" s="9"/>
-      <c r="G68" s="9"/>
+      <c r="A68" s="6"/>
+      <c r="B68" s="6"/>
+      <c r="C68" s="6"/>
+      <c r="D68" s="6"/>
+      <c r="E68" s="6"/>
+      <c r="F68" s="6"/>
+      <c r="G68" s="6"/>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A69" s="9"/>
-      <c r="B69" s="9"/>
-      <c r="C69" s="9"/>
-      <c r="D69" s="9"/>
-      <c r="E69" s="9"/>
-      <c r="F69" s="9"/>
-      <c r="G69" s="9"/>
+      <c r="A69" s="6"/>
+      <c r="B69" s="6"/>
+      <c r="C69" s="6"/>
+      <c r="D69" s="6"/>
+      <c r="E69" s="6"/>
+      <c r="F69" s="6"/>
+      <c r="G69" s="6"/>
     </row>
     <row r="70" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A70" s="9"/>
-      <c r="B70" s="9"/>
-      <c r="C70" s="9"/>
-      <c r="D70" s="9"/>
-      <c r="E70" s="9"/>
-      <c r="F70" s="9"/>
-      <c r="G70" s="9"/>
+      <c r="A70" s="6"/>
+      <c r="B70" s="6"/>
+      <c r="C70" s="6"/>
+      <c r="D70" s="6"/>
+      <c r="E70" s="6"/>
+      <c r="F70" s="6"/>
+      <c r="G70" s="6"/>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A71" s="9"/>
-      <c r="B71" s="9"/>
-      <c r="C71" s="9"/>
-      <c r="D71" s="9"/>
-      <c r="E71" s="9"/>
-      <c r="F71" s="9"/>
-      <c r="G71" s="9"/>
+      <c r="A71" s="6"/>
+      <c r="B71" s="6"/>
+      <c r="C71" s="6"/>
+      <c r="D71" s="6"/>
+      <c r="E71" s="6"/>
+      <c r="F71" s="6"/>
+      <c r="G71" s="6"/>
     </row>
     <row r="72" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A72" s="9"/>
-      <c r="B72" s="9"/>
-      <c r="C72" s="9"/>
-      <c r="D72" s="9"/>
-      <c r="E72" s="9"/>
-      <c r="F72" s="9"/>
-      <c r="G72" s="9"/>
+      <c r="A72" s="6"/>
+      <c r="B72" s="6"/>
+      <c r="C72" s="6"/>
+      <c r="D72" s="6"/>
+      <c r="E72" s="6"/>
+      <c r="F72" s="6"/>
+      <c r="G72" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="C29:F29"/>
+    <mergeCell ref="C28:F28"/>
+    <mergeCell ref="C35:F35"/>
+    <mergeCell ref="C36:F36"/>
+    <mergeCell ref="C32:F32"/>
+    <mergeCell ref="C30:F30"/>
+    <mergeCell ref="C33:F33"/>
     <mergeCell ref="A40:F49"/>
     <mergeCell ref="A53:G72"/>
     <mergeCell ref="A31:B31"/>
@@ -1794,16 +2279,6 @@
     <mergeCell ref="A35:B35"/>
     <mergeCell ref="A36:B36"/>
     <mergeCell ref="C34:F34"/>
-    <mergeCell ref="C29:F29"/>
-    <mergeCell ref="C28:F28"/>
-    <mergeCell ref="C35:F35"/>
-    <mergeCell ref="C36:F36"/>
-    <mergeCell ref="C32:F32"/>
-    <mergeCell ref="C30:F30"/>
-    <mergeCell ref="C33:F33"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="A30:B30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1811,36 +2286,2416 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B8526C6-7212-EE4B-BB25-602DDD881251}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:L70"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="22.1640625" customWidth="1"/>
+    <col min="4" max="4" width="19.6640625" customWidth="1"/>
+    <col min="5" max="5" width="24.83203125" customWidth="1"/>
+    <col min="6" max="6" width="20.83203125" customWidth="1"/>
+    <col min="7" max="7" width="21.33203125" customWidth="1"/>
+    <col min="8" max="8" width="20.1640625" customWidth="1"/>
+    <col min="9" max="9" width="40.83203125" customWidth="1"/>
+    <col min="10" max="10" width="32.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" s="15" t="s">
+        <v>85</v>
+      </c>
+      <c r="E1" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="G1" s="16" t="s">
+        <v>100</v>
+      </c>
+      <c r="H1" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="I1" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" s="15" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G2">
+        <v>12</v>
+      </c>
+      <c r="H2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G3">
+        <v>12</v>
+      </c>
+      <c r="H3" t="s">
+        <v>9</v>
+      </c>
+      <c r="I3" t="s">
+        <v>38</v>
+      </c>
+      <c r="J3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4">
+        <v>12</v>
+      </c>
+      <c r="H4" t="s">
+        <v>9</v>
+      </c>
+      <c r="I4" t="s">
+        <v>86</v>
+      </c>
+      <c r="J4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" t="s">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I5" t="s">
+        <v>42</v>
+      </c>
+      <c r="J5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>87</v>
+      </c>
+      <c r="C6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" t="s">
+        <v>8</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I6" t="s">
+        <v>102</v>
+      </c>
+      <c r="J6" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>88</v>
+      </c>
+      <c r="C7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7" t="s">
+        <v>27</v>
+      </c>
+      <c r="I7" t="s">
+        <v>104</v>
+      </c>
+      <c r="J7" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>89</v>
+      </c>
+      <c r="C8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>8</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8" t="s">
+        <v>27</v>
+      </c>
+      <c r="I8" t="s">
+        <v>105</v>
+      </c>
+      <c r="J8" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>90</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9" t="s">
+        <v>8</v>
+      </c>
+      <c r="F9" t="s">
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9" t="s">
+        <v>11</v>
+      </c>
+      <c r="I9" t="s">
+        <v>106</v>
+      </c>
+      <c r="J9" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10" t="s">
+        <v>24</v>
+      </c>
+      <c r="D10" t="s">
+        <v>8</v>
+      </c>
+      <c r="E10" t="s">
+        <v>8</v>
+      </c>
+      <c r="F10" t="s">
+        <v>0</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10" t="s">
+        <v>11</v>
+      </c>
+      <c r="I10" t="s">
+        <v>108</v>
+      </c>
+      <c r="J10" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>92</v>
+      </c>
+      <c r="C11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11" t="s">
+        <v>8</v>
+      </c>
+      <c r="E11" t="s">
+        <v>8</v>
+      </c>
+      <c r="F11" t="s">
+        <v>0</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11" t="s">
+        <v>11</v>
+      </c>
+      <c r="I11" t="s">
+        <v>109</v>
+      </c>
+      <c r="J11" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>93</v>
+      </c>
+      <c r="C12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" t="s">
+        <v>0</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>8</v>
+      </c>
+      <c r="G12">
+        <v>12</v>
+      </c>
+      <c r="H12" t="s">
+        <v>9</v>
+      </c>
+      <c r="I12" t="s">
+        <v>110</v>
+      </c>
+      <c r="J12" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" t="s">
+        <v>16</v>
+      </c>
+      <c r="D13" t="s">
+        <v>0</v>
+      </c>
+      <c r="E13" t="s">
+        <v>8</v>
+      </c>
+      <c r="F13" t="s">
+        <v>8</v>
+      </c>
+      <c r="G13">
+        <v>12</v>
+      </c>
+      <c r="H13" t="s">
+        <v>9</v>
+      </c>
+      <c r="I13" t="s">
+        <v>94</v>
+      </c>
+      <c r="J13" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="11"/>
+    </row>
+    <row r="15" spans="1:10" ht="32" x14ac:dyDescent="0.4">
+      <c r="A15" s="11" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A17" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>96</v>
+      </c>
+      <c r="B18">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>70</v>
+      </c>
+      <c r="B19" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>72</v>
+      </c>
+      <c r="B20" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>74</v>
+      </c>
+      <c r="B21" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>116</v>
+      </c>
+      <c r="B22" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>97</v>
+      </c>
+      <c r="B23" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>118</v>
+      </c>
+      <c r="B24" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>98</v>
+      </c>
+      <c r="B25" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" ht="32" x14ac:dyDescent="0.4">
+      <c r="A27" s="11" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A28" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="B28" s="6"/>
+      <c r="C28" s="6"/>
+      <c r="D28" s="6"/>
+      <c r="E28" s="6"/>
+      <c r="F28" s="6"/>
+      <c r="G28" s="6"/>
+      <c r="H28" s="6"/>
+      <c r="I28" s="6"/>
+      <c r="J28" s="6"/>
+      <c r="K28" s="6"/>
+      <c r="L28" s="6"/>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A29" s="6"/>
+      <c r="B29" s="6"/>
+      <c r="C29" s="6"/>
+      <c r="D29" s="6"/>
+      <c r="E29" s="6"/>
+      <c r="F29" s="6"/>
+      <c r="G29" s="6"/>
+      <c r="H29" s="6"/>
+      <c r="I29" s="6"/>
+      <c r="J29" s="6"/>
+      <c r="K29" s="6"/>
+      <c r="L29" s="6"/>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A30" s="6"/>
+      <c r="B30" s="6"/>
+      <c r="C30" s="6"/>
+      <c r="D30" s="6"/>
+      <c r="E30" s="6"/>
+      <c r="F30" s="6"/>
+      <c r="G30" s="6"/>
+      <c r="H30" s="6"/>
+      <c r="I30" s="6"/>
+      <c r="J30" s="6"/>
+      <c r="K30" s="6"/>
+      <c r="L30" s="6"/>
+    </row>
+    <row r="31" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="6"/>
+      <c r="B31" s="6"/>
+      <c r="C31" s="6"/>
+      <c r="D31" s="6"/>
+      <c r="E31" s="6"/>
+      <c r="F31" s="6"/>
+      <c r="G31" s="6"/>
+      <c r="H31" s="6"/>
+      <c r="I31" s="6"/>
+      <c r="J31" s="6"/>
+      <c r="K31" s="6"/>
+      <c r="L31" s="6"/>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A32" s="6"/>
+      <c r="B32" s="6"/>
+      <c r="C32" s="6"/>
+      <c r="D32" s="6"/>
+      <c r="E32" s="6"/>
+      <c r="F32" s="6"/>
+      <c r="G32" s="6"/>
+      <c r="H32" s="6"/>
+      <c r="I32" s="6"/>
+      <c r="J32" s="6"/>
+      <c r="K32" s="6"/>
+      <c r="L32" s="6"/>
+    </row>
+    <row r="33" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="6"/>
+      <c r="B33" s="6"/>
+      <c r="C33" s="6"/>
+      <c r="D33" s="6"/>
+      <c r="E33" s="6"/>
+      <c r="F33" s="6"/>
+      <c r="G33" s="6"/>
+      <c r="H33" s="6"/>
+      <c r="I33" s="6"/>
+      <c r="J33" s="6"/>
+      <c r="K33" s="6"/>
+      <c r="L33" s="6"/>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A34" s="6"/>
+      <c r="B34" s="6"/>
+      <c r="C34" s="6"/>
+      <c r="D34" s="6"/>
+      <c r="E34" s="6"/>
+      <c r="F34" s="6"/>
+      <c r="G34" s="6"/>
+      <c r="H34" s="6"/>
+      <c r="I34" s="6"/>
+      <c r="J34" s="6"/>
+      <c r="K34" s="6"/>
+      <c r="L34" s="6"/>
+    </row>
+    <row r="35" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="6"/>
+      <c r="B35" s="6"/>
+      <c r="C35" s="6"/>
+      <c r="D35" s="6"/>
+      <c r="E35" s="6"/>
+      <c r="F35" s="6"/>
+      <c r="G35" s="6"/>
+      <c r="H35" s="6"/>
+      <c r="I35" s="6"/>
+      <c r="J35" s="6"/>
+      <c r="K35" s="6"/>
+      <c r="L35" s="6"/>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A36" s="6"/>
+      <c r="B36" s="6"/>
+      <c r="C36" s="6"/>
+      <c r="D36" s="6"/>
+      <c r="E36" s="6"/>
+      <c r="F36" s="6"/>
+      <c r="G36" s="6"/>
+      <c r="H36" s="6"/>
+      <c r="I36" s="6"/>
+      <c r="J36" s="6"/>
+      <c r="K36" s="6"/>
+      <c r="L36" s="6"/>
+    </row>
+    <row r="37" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="6"/>
+      <c r="B37" s="6"/>
+      <c r="C37" s="6"/>
+      <c r="D37" s="6"/>
+      <c r="E37" s="6"/>
+      <c r="F37" s="6"/>
+      <c r="G37" s="6"/>
+      <c r="H37" s="6"/>
+      <c r="I37" s="6"/>
+      <c r="J37" s="6"/>
+      <c r="K37" s="6"/>
+      <c r="L37" s="6"/>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A38" s="6"/>
+      <c r="B38" s="6"/>
+      <c r="C38" s="6"/>
+      <c r="D38" s="6"/>
+      <c r="E38" s="6"/>
+      <c r="F38" s="6"/>
+      <c r="G38" s="6"/>
+      <c r="H38" s="6"/>
+      <c r="I38" s="6"/>
+      <c r="J38" s="6"/>
+      <c r="K38" s="6"/>
+      <c r="L38" s="6"/>
+    </row>
+    <row r="41" spans="1:12" ht="32" x14ac:dyDescent="0.4">
+      <c r="A41" s="17" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A42" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="B42" s="18"/>
+      <c r="C42" s="18"/>
+      <c r="D42" s="18"/>
+      <c r="E42" s="18"/>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A43" s="18"/>
+      <c r="B43" s="18"/>
+      <c r="C43" s="18"/>
+      <c r="D43" s="18"/>
+      <c r="E43" s="18"/>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A44" s="18"/>
+      <c r="B44" s="18"/>
+      <c r="C44" s="18"/>
+      <c r="D44" s="18"/>
+      <c r="E44" s="18"/>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A45" s="18"/>
+      <c r="B45" s="18"/>
+      <c r="C45" s="18"/>
+      <c r="D45" s="18"/>
+      <c r="E45" s="18"/>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A46" s="18"/>
+      <c r="B46" s="18"/>
+      <c r="C46" s="18"/>
+      <c r="D46" s="18"/>
+      <c r="E46" s="18"/>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A47" s="18"/>
+      <c r="B47" s="18"/>
+      <c r="C47" s="18"/>
+      <c r="D47" s="18"/>
+      <c r="E47" s="18"/>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A48" s="18"/>
+      <c r="B48" s="18"/>
+      <c r="C48" s="18"/>
+      <c r="D48" s="18"/>
+      <c r="E48" s="18"/>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A49" s="18"/>
+      <c r="B49" s="18"/>
+      <c r="C49" s="18"/>
+      <c r="D49" s="18"/>
+      <c r="E49" s="18"/>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A50" s="18"/>
+      <c r="B50" s="18"/>
+      <c r="C50" s="18"/>
+      <c r="D50" s="18"/>
+      <c r="E50" s="18"/>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A51" s="18"/>
+      <c r="B51" s="18"/>
+      <c r="C51" s="18"/>
+      <c r="D51" s="18"/>
+      <c r="E51" s="18"/>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A52" s="18"/>
+      <c r="B52" s="18"/>
+      <c r="C52" s="18"/>
+      <c r="D52" s="18"/>
+      <c r="E52" s="18"/>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A53" s="18"/>
+      <c r="B53" s="18"/>
+      <c r="C53" s="18"/>
+      <c r="D53" s="18"/>
+      <c r="E53" s="18"/>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A54" s="18"/>
+      <c r="B54" s="18"/>
+      <c r="C54" s="18"/>
+      <c r="D54" s="18"/>
+      <c r="E54" s="18"/>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A55" s="18"/>
+      <c r="B55" s="18"/>
+      <c r="C55" s="18"/>
+      <c r="D55" s="18"/>
+      <c r="E55" s="18"/>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A56" s="18"/>
+      <c r="B56" s="18"/>
+      <c r="C56" s="18"/>
+      <c r="D56" s="18"/>
+      <c r="E56" s="18"/>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A57" s="18"/>
+      <c r="B57" s="18"/>
+      <c r="C57" s="18"/>
+      <c r="D57" s="18"/>
+      <c r="E57" s="18"/>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A58" s="18"/>
+      <c r="B58" s="18"/>
+      <c r="C58" s="18"/>
+      <c r="D58" s="18"/>
+      <c r="E58" s="18"/>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A59" s="18"/>
+      <c r="B59" s="18"/>
+      <c r="C59" s="18"/>
+      <c r="D59" s="18"/>
+      <c r="E59" s="18"/>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A60" s="18"/>
+      <c r="B60" s="18"/>
+      <c r="C60" s="18"/>
+      <c r="D60" s="18"/>
+      <c r="E60" s="18"/>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A61" s="18"/>
+      <c r="B61" s="18"/>
+      <c r="C61" s="18"/>
+      <c r="D61" s="18"/>
+      <c r="E61" s="18"/>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A62" s="18"/>
+      <c r="B62" s="18"/>
+      <c r="C62" s="18"/>
+      <c r="D62" s="18"/>
+      <c r="E62" s="18"/>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A63" s="18"/>
+      <c r="B63" s="18"/>
+      <c r="C63" s="18"/>
+      <c r="D63" s="18"/>
+      <c r="E63" s="18"/>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A64" s="18"/>
+      <c r="B64" s="18"/>
+      <c r="C64" s="18"/>
+      <c r="D64" s="18"/>
+      <c r="E64" s="18"/>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A65" s="18"/>
+      <c r="B65" s="18"/>
+      <c r="C65" s="18"/>
+      <c r="D65" s="18"/>
+      <c r="E65" s="18"/>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A66" s="18"/>
+      <c r="B66" s="18"/>
+      <c r="C66" s="18"/>
+      <c r="D66" s="18"/>
+      <c r="E66" s="18"/>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A67" s="18"/>
+      <c r="B67" s="18"/>
+      <c r="C67" s="18"/>
+      <c r="D67" s="18"/>
+      <c r="E67" s="18"/>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A68" s="18"/>
+      <c r="B68" s="18"/>
+      <c r="C68" s="18"/>
+      <c r="D68" s="18"/>
+      <c r="E68" s="18"/>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A69" s="18"/>
+      <c r="B69" s="18"/>
+      <c r="C69" s="18"/>
+      <c r="D69" s="18"/>
+      <c r="E69" s="18"/>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A70" s="18"/>
+      <c r="B70" s="18"/>
+      <c r="C70" s="18"/>
+      <c r="D70" s="18"/>
+      <c r="E70" s="18"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A28:L38"/>
+    <mergeCell ref="A42:E70"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9647CE43-ED5F-CF49-B719-99CBC527DB3E}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:J64"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="25.83203125" customWidth="1"/>
+    <col min="4" max="4" width="21" customWidth="1"/>
+    <col min="5" max="5" width="23.1640625" customWidth="1"/>
+    <col min="6" max="6" width="15" customWidth="1"/>
+    <col min="8" max="8" width="13.33203125" customWidth="1"/>
+    <col min="9" max="9" width="42.5" customWidth="1"/>
+    <col min="10" max="10" width="32.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="31" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="E1" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" s="16" t="s">
+        <v>138</v>
+      </c>
+      <c r="G1" s="16" t="s">
+        <v>139</v>
+      </c>
+      <c r="H1" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="I1" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" s="15" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G2">
+        <v>12</v>
+      </c>
+      <c r="H2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G3">
+        <v>12</v>
+      </c>
+      <c r="H3" t="s">
+        <v>9</v>
+      </c>
+      <c r="I3" t="s">
+        <v>38</v>
+      </c>
+      <c r="J3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4">
+        <v>12</v>
+      </c>
+      <c r="H4" t="s">
+        <v>9</v>
+      </c>
+      <c r="I4" t="s">
+        <v>94</v>
+      </c>
+      <c r="J4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G5">
+        <v>12</v>
+      </c>
+      <c r="H5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I5" t="s">
+        <v>124</v>
+      </c>
+      <c r="J5" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>93</v>
+      </c>
+      <c r="C6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" t="s">
+        <v>8</v>
+      </c>
+      <c r="G6">
+        <v>12</v>
+      </c>
+      <c r="H6" t="s">
+        <v>9</v>
+      </c>
+      <c r="I6" t="s">
+        <v>125</v>
+      </c>
+      <c r="J6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>126</v>
+      </c>
+      <c r="C7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" t="s">
+        <v>0</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7" t="s">
+        <v>11</v>
+      </c>
+      <c r="I7" t="s">
+        <v>127</v>
+      </c>
+      <c r="J7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>129</v>
+      </c>
+      <c r="C8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>0</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8" t="s">
+        <v>11</v>
+      </c>
+      <c r="I8" t="s">
+        <v>130</v>
+      </c>
+      <c r="J8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>131</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9" t="s">
+        <v>8</v>
+      </c>
+      <c r="F9" t="s">
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9" t="s">
+        <v>11</v>
+      </c>
+      <c r="I9" t="s">
+        <v>132</v>
+      </c>
+      <c r="J9" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" t="s">
+        <v>0</v>
+      </c>
+      <c r="E10" t="s">
+        <v>8</v>
+      </c>
+      <c r="F10" t="s">
+        <v>0</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10" t="s">
+        <v>11</v>
+      </c>
+      <c r="I10" t="s">
+        <v>133</v>
+      </c>
+      <c r="J10" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>134</v>
+      </c>
+      <c r="C11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11" t="s">
+        <v>0</v>
+      </c>
+      <c r="E11" t="s">
+        <v>8</v>
+      </c>
+      <c r="F11" t="s">
+        <v>0</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11" t="s">
+        <v>11</v>
+      </c>
+      <c r="I11" t="s">
+        <v>135</v>
+      </c>
+      <c r="J11" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>136</v>
+      </c>
+      <c r="C12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" t="s">
+        <v>0</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>8</v>
+      </c>
+      <c r="G12">
+        <v>12</v>
+      </c>
+      <c r="H12" t="s">
+        <v>9</v>
+      </c>
+      <c r="I12" t="s">
+        <v>94</v>
+      </c>
+      <c r="J12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>137</v>
+      </c>
+      <c r="C13" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" t="s">
+        <v>0</v>
+      </c>
+      <c r="E13" t="s">
+        <v>8</v>
+      </c>
+      <c r="F13" t="s">
+        <v>8</v>
+      </c>
+      <c r="G13">
+        <v>12</v>
+      </c>
+      <c r="H13" t="s">
+        <v>9</v>
+      </c>
+      <c r="I13" t="s">
+        <v>94</v>
+      </c>
+      <c r="J13" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="32" x14ac:dyDescent="0.4">
+      <c r="A16" s="11" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A18" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>141</v>
+      </c>
+      <c r="B19">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>70</v>
+      </c>
+      <c r="B20" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>72</v>
+      </c>
+      <c r="B21" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>74</v>
+      </c>
+      <c r="B22" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>77</v>
+      </c>
+      <c r="B23" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>146</v>
+      </c>
+      <c r="B24" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>147</v>
+      </c>
+      <c r="B25" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>148</v>
+      </c>
+      <c r="B26" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="32" x14ac:dyDescent="0.4">
+      <c r="A29" s="17" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A30" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="B30" s="18"/>
+      <c r="C30" s="18"/>
+      <c r="D30" s="18"/>
+      <c r="E30" s="18"/>
+      <c r="F30" s="18"/>
+      <c r="G30" s="18"/>
+      <c r="H30" s="18"/>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A31" s="18"/>
+      <c r="B31" s="18"/>
+      <c r="C31" s="18"/>
+      <c r="D31" s="18"/>
+      <c r="E31" s="18"/>
+      <c r="F31" s="18"/>
+      <c r="G31" s="18"/>
+      <c r="H31" s="18"/>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A32" s="18"/>
+      <c r="B32" s="18"/>
+      <c r="C32" s="18"/>
+      <c r="D32" s="18"/>
+      <c r="E32" s="18"/>
+      <c r="F32" s="18"/>
+      <c r="G32" s="18"/>
+      <c r="H32" s="18"/>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A33" s="18"/>
+      <c r="B33" s="18"/>
+      <c r="C33" s="18"/>
+      <c r="D33" s="18"/>
+      <c r="E33" s="18"/>
+      <c r="F33" s="18"/>
+      <c r="G33" s="18"/>
+      <c r="H33" s="18"/>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A34" s="18"/>
+      <c r="B34" s="18"/>
+      <c r="C34" s="18"/>
+      <c r="D34" s="18"/>
+      <c r="E34" s="18"/>
+      <c r="F34" s="18"/>
+      <c r="G34" s="18"/>
+      <c r="H34" s="18"/>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A35" s="18"/>
+      <c r="B35" s="18"/>
+      <c r="C35" s="18"/>
+      <c r="D35" s="18"/>
+      <c r="E35" s="18"/>
+      <c r="F35" s="18"/>
+      <c r="G35" s="18"/>
+      <c r="H35" s="18"/>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A36" s="18"/>
+      <c r="B36" s="18"/>
+      <c r="C36" s="18"/>
+      <c r="D36" s="18"/>
+      <c r="E36" s="18"/>
+      <c r="F36" s="18"/>
+      <c r="G36" s="18"/>
+      <c r="H36" s="18"/>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A37" s="18"/>
+      <c r="B37" s="18"/>
+      <c r="C37" s="18"/>
+      <c r="D37" s="18"/>
+      <c r="E37" s="18"/>
+      <c r="F37" s="18"/>
+      <c r="G37" s="18"/>
+      <c r="H37" s="18"/>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A38" s="18"/>
+      <c r="B38" s="18"/>
+      <c r="C38" s="18"/>
+      <c r="D38" s="18"/>
+      <c r="E38" s="18"/>
+      <c r="F38" s="18"/>
+      <c r="G38" s="18"/>
+      <c r="H38" s="18"/>
+    </row>
+    <row r="41" spans="1:8" ht="32" x14ac:dyDescent="0.4">
+      <c r="A41" s="17" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A42" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="B42" s="18"/>
+      <c r="C42" s="18"/>
+      <c r="D42" s="18"/>
+      <c r="E42" s="18"/>
+      <c r="F42" s="18"/>
+      <c r="G42" s="18"/>
+      <c r="H42" s="18"/>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A43" s="18"/>
+      <c r="B43" s="18"/>
+      <c r="C43" s="18"/>
+      <c r="D43" s="18"/>
+      <c r="E43" s="18"/>
+      <c r="F43" s="18"/>
+      <c r="G43" s="18"/>
+      <c r="H43" s="18"/>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A44" s="18"/>
+      <c r="B44" s="18"/>
+      <c r="C44" s="18"/>
+      <c r="D44" s="18"/>
+      <c r="E44" s="18"/>
+      <c r="F44" s="18"/>
+      <c r="G44" s="18"/>
+      <c r="H44" s="18"/>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A45" s="18"/>
+      <c r="B45" s="18"/>
+      <c r="C45" s="18"/>
+      <c r="D45" s="18"/>
+      <c r="E45" s="18"/>
+      <c r="F45" s="18"/>
+      <c r="G45" s="18"/>
+      <c r="H45" s="18"/>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A46" s="18"/>
+      <c r="B46" s="18"/>
+      <c r="C46" s="18"/>
+      <c r="D46" s="18"/>
+      <c r="E46" s="18"/>
+      <c r="F46" s="18"/>
+      <c r="G46" s="18"/>
+      <c r="H46" s="18"/>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A47" s="18"/>
+      <c r="B47" s="18"/>
+      <c r="C47" s="18"/>
+      <c r="D47" s="18"/>
+      <c r="E47" s="18"/>
+      <c r="F47" s="18"/>
+      <c r="G47" s="18"/>
+      <c r="H47" s="18"/>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A48" s="18"/>
+      <c r="B48" s="18"/>
+      <c r="C48" s="18"/>
+      <c r="D48" s="18"/>
+      <c r="E48" s="18"/>
+      <c r="F48" s="18"/>
+      <c r="G48" s="18"/>
+      <c r="H48" s="18"/>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A49" s="18"/>
+      <c r="B49" s="18"/>
+      <c r="C49" s="18"/>
+      <c r="D49" s="18"/>
+      <c r="E49" s="18"/>
+      <c r="F49" s="18"/>
+      <c r="G49" s="18"/>
+      <c r="H49" s="18"/>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A50" s="18"/>
+      <c r="B50" s="18"/>
+      <c r="C50" s="18"/>
+      <c r="D50" s="18"/>
+      <c r="E50" s="18"/>
+      <c r="F50" s="18"/>
+      <c r="G50" s="18"/>
+      <c r="H50" s="18"/>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A51" s="18"/>
+      <c r="B51" s="18"/>
+      <c r="C51" s="18"/>
+      <c r="D51" s="18"/>
+      <c r="E51" s="18"/>
+      <c r="F51" s="18"/>
+      <c r="G51" s="18"/>
+      <c r="H51" s="18"/>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A52" s="18"/>
+      <c r="B52" s="18"/>
+      <c r="C52" s="18"/>
+      <c r="D52" s="18"/>
+      <c r="E52" s="18"/>
+      <c r="F52" s="18"/>
+      <c r="G52" s="18"/>
+      <c r="H52" s="18"/>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A53" s="18"/>
+      <c r="B53" s="18"/>
+      <c r="C53" s="18"/>
+      <c r="D53" s="18"/>
+      <c r="E53" s="18"/>
+      <c r="F53" s="18"/>
+      <c r="G53" s="18"/>
+      <c r="H53" s="18"/>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A54" s="18"/>
+      <c r="B54" s="18"/>
+      <c r="C54" s="18"/>
+      <c r="D54" s="18"/>
+      <c r="E54" s="18"/>
+      <c r="F54" s="18"/>
+      <c r="G54" s="18"/>
+      <c r="H54" s="18"/>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A55" s="18"/>
+      <c r="B55" s="18"/>
+      <c r="C55" s="18"/>
+      <c r="D55" s="18"/>
+      <c r="E55" s="18"/>
+      <c r="F55" s="18"/>
+      <c r="G55" s="18"/>
+      <c r="H55" s="18"/>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A56" s="18"/>
+      <c r="B56" s="18"/>
+      <c r="C56" s="18"/>
+      <c r="D56" s="18"/>
+      <c r="E56" s="18"/>
+      <c r="F56" s="18"/>
+      <c r="G56" s="18"/>
+      <c r="H56" s="18"/>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A57" s="18"/>
+      <c r="B57" s="18"/>
+      <c r="C57" s="18"/>
+      <c r="D57" s="18"/>
+      <c r="E57" s="18"/>
+      <c r="F57" s="18"/>
+      <c r="G57" s="18"/>
+      <c r="H57" s="18"/>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A58" s="18"/>
+      <c r="B58" s="18"/>
+      <c r="C58" s="18"/>
+      <c r="D58" s="18"/>
+      <c r="E58" s="18"/>
+      <c r="F58" s="18"/>
+      <c r="G58" s="18"/>
+      <c r="H58" s="18"/>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A59" s="18"/>
+      <c r="B59" s="18"/>
+      <c r="C59" s="18"/>
+      <c r="D59" s="18"/>
+      <c r="E59" s="18"/>
+      <c r="F59" s="18"/>
+      <c r="G59" s="18"/>
+      <c r="H59" s="18"/>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A60" s="18"/>
+      <c r="B60" s="18"/>
+      <c r="C60" s="18"/>
+      <c r="D60" s="18"/>
+      <c r="E60" s="18"/>
+      <c r="F60" s="18"/>
+      <c r="G60" s="18"/>
+      <c r="H60" s="18"/>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A61" s="18"/>
+      <c r="B61" s="18"/>
+      <c r="C61" s="18"/>
+      <c r="D61" s="18"/>
+      <c r="E61" s="18"/>
+      <c r="F61" s="18"/>
+      <c r="G61" s="18"/>
+      <c r="H61" s="18"/>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A62" s="18"/>
+      <c r="B62" s="18"/>
+      <c r="C62" s="18"/>
+      <c r="D62" s="18"/>
+      <c r="E62" s="18"/>
+      <c r="F62" s="18"/>
+      <c r="G62" s="18"/>
+      <c r="H62" s="18"/>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A63" s="18"/>
+      <c r="B63" s="18"/>
+      <c r="C63" s="18"/>
+      <c r="D63" s="18"/>
+      <c r="E63" s="18"/>
+      <c r="F63" s="18"/>
+      <c r="G63" s="18"/>
+      <c r="H63" s="18"/>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A64" s="18"/>
+      <c r="B64" s="18"/>
+      <c r="C64" s="18"/>
+      <c r="D64" s="18"/>
+      <c r="E64" s="18"/>
+      <c r="F64" s="18"/>
+      <c r="G64" s="18"/>
+      <c r="H64" s="18"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A30:H38"/>
+    <mergeCell ref="A42:H64"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CC2A96B-595B-E747-BF11-6EEB10631C05}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="19" customWidth="1"/>
+    <col min="3" max="3" width="18.5" customWidth="1"/>
+    <col min="4" max="4" width="37" customWidth="1"/>
+    <col min="5" max="5" width="29.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="15" t="s">
+        <v>151</v>
+      </c>
+      <c r="B1" s="15" t="s">
+        <v>152</v>
+      </c>
+      <c r="C1" s="15" t="s">
+        <v>153</v>
+      </c>
+      <c r="D1" s="15" t="s">
+        <v>154</v>
+      </c>
+      <c r="E1" s="15" t="s">
+        <v>155</v>
+      </c>
+      <c r="F1" s="19"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>156</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>157</v>
+      </c>
+      <c r="D2" t="s">
+        <v>158</v>
+      </c>
+      <c r="E2" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>156</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
+        <v>157</v>
+      </c>
+      <c r="D3" t="s">
+        <v>160</v>
+      </c>
+      <c r="E3" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>156</v>
+      </c>
+      <c r="B4" t="s">
+        <v>134</v>
+      </c>
+      <c r="C4" t="s">
+        <v>157</v>
+      </c>
+      <c r="D4" t="s">
+        <v>161</v>
+      </c>
+      <c r="E4" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>156</v>
+      </c>
+      <c r="B5" t="s">
+        <v>162</v>
+      </c>
+      <c r="C5" t="s">
+        <v>157</v>
+      </c>
+      <c r="D5" t="s">
+        <v>163</v>
+      </c>
+      <c r="E5" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>164</v>
+      </c>
+      <c r="B6" t="s">
+        <v>90</v>
+      </c>
+      <c r="C6" t="s">
+        <v>157</v>
+      </c>
+      <c r="D6" t="s">
+        <v>165</v>
+      </c>
+      <c r="E6" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>164</v>
+      </c>
+      <c r="B7" t="s">
+        <v>91</v>
+      </c>
+      <c r="C7" t="s">
+        <v>157</v>
+      </c>
+      <c r="D7" t="s">
+        <v>167</v>
+      </c>
+      <c r="E7" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>164</v>
+      </c>
+      <c r="B8" t="s">
+        <v>92</v>
+      </c>
+      <c r="C8" t="s">
+        <v>157</v>
+      </c>
+      <c r="D8" t="s">
+        <v>168</v>
+      </c>
+      <c r="E8" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>169</v>
+      </c>
+      <c r="B9" t="s">
+        <v>126</v>
+      </c>
+      <c r="C9" t="s">
+        <v>157</v>
+      </c>
+      <c r="D9" t="s">
+        <v>170</v>
+      </c>
+      <c r="E9" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>169</v>
+      </c>
+      <c r="B10" t="s">
+        <v>129</v>
+      </c>
+      <c r="C10" t="s">
+        <v>157</v>
+      </c>
+      <c r="D10" t="s">
+        <v>172</v>
+      </c>
+      <c r="E10" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>169</v>
+      </c>
+      <c r="B11" t="s">
+        <v>131</v>
+      </c>
+      <c r="C11" t="s">
+        <v>157</v>
+      </c>
+      <c r="D11" t="s">
+        <v>173</v>
+      </c>
+      <c r="E11" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="32" x14ac:dyDescent="0.4">
+      <c r="A14" s="11" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A16" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>175</v>
+      </c>
+      <c r="B17">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>176</v>
+      </c>
+      <c r="B18">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>177</v>
+      </c>
+      <c r="B19">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>178</v>
+      </c>
+      <c r="B20">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>79</v>
+      </c>
+      <c r="B21" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>97</v>
+      </c>
+      <c r="B22" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>146</v>
+      </c>
+      <c r="B23" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="32" x14ac:dyDescent="0.4">
+      <c r="A26" s="11" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="28" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="12" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="30" spans="1:2" ht="17" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="12" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="32" spans="1:2" ht="17" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="12" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" ht="16" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="34" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="12" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" ht="16" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="36" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="12" t="s">
+        <v>183</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B924726-B2AB-6640-9A1C-88ACA9E2EEDE}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="21.5" customWidth="1"/>
+    <col min="3" max="4" width="23.6640625" customWidth="1"/>
+    <col min="5" max="5" width="29.5" customWidth="1"/>
+    <col min="6" max="6" width="26.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="15" t="s">
+        <v>184</v>
+      </c>
+      <c r="D1" s="15" t="s">
+        <v>185</v>
+      </c>
+      <c r="E1" s="15" t="s">
+        <v>186</v>
+      </c>
+      <c r="F1" s="15" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>156</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" t="s">
+        <v>187</v>
+      </c>
+      <c r="F2" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>156</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E3" t="s">
+        <v>187</v>
+      </c>
+      <c r="F3" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>156</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s">
+        <v>189</v>
+      </c>
+      <c r="D4" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" t="s">
+        <v>187</v>
+      </c>
+      <c r="F4" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>156</v>
+      </c>
+      <c r="B5" t="s">
+        <v>78</v>
+      </c>
+      <c r="C5" t="s">
+        <v>189</v>
+      </c>
+      <c r="D5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" t="s">
+        <v>187</v>
+      </c>
+      <c r="F5" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>164</v>
+      </c>
+      <c r="B6" t="s">
+        <v>87</v>
+      </c>
+      <c r="C6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" t="s">
+        <v>192</v>
+      </c>
+      <c r="F6" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>164</v>
+      </c>
+      <c r="B7" t="s">
+        <v>90</v>
+      </c>
+      <c r="C7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" t="s">
+        <v>0</v>
+      </c>
+      <c r="E7" t="s">
+        <v>187</v>
+      </c>
+      <c r="F7" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>164</v>
+      </c>
+      <c r="B8" t="s">
+        <v>91</v>
+      </c>
+      <c r="C8" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" t="s">
+        <v>0</v>
+      </c>
+      <c r="E8" t="s">
+        <v>187</v>
+      </c>
+      <c r="F8" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>164</v>
+      </c>
+      <c r="B9" t="s">
+        <v>92</v>
+      </c>
+      <c r="C9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" t="s">
+        <v>0</v>
+      </c>
+      <c r="E9" t="s">
+        <v>187</v>
+      </c>
+      <c r="F9" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>169</v>
+      </c>
+      <c r="B10" t="s">
+        <v>126</v>
+      </c>
+      <c r="C10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10" t="s">
+        <v>0</v>
+      </c>
+      <c r="E10" t="s">
+        <v>187</v>
+      </c>
+      <c r="F10" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>169</v>
+      </c>
+      <c r="B11" t="s">
+        <v>129</v>
+      </c>
+      <c r="C11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D11" t="s">
+        <v>0</v>
+      </c>
+      <c r="E11" t="s">
+        <v>187</v>
+      </c>
+      <c r="F11" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>169</v>
+      </c>
+      <c r="B12" t="s">
+        <v>131</v>
+      </c>
+      <c r="C12" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" t="s">
+        <v>0</v>
+      </c>
+      <c r="E12" t="s">
+        <v>187</v>
+      </c>
+      <c r="F12" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="32" x14ac:dyDescent="0.4">
+      <c r="A15" s="11" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>197</v>
+      </c>
+      <c r="B18" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>199</v>
+      </c>
+      <c r="B19" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>201</v>
+      </c>
+      <c r="B20" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>203</v>
+      </c>
+      <c r="B21" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>205</v>
+      </c>
+      <c r="B22" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>207</v>
+      </c>
+      <c r="B23" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="32" x14ac:dyDescent="0.4">
+      <c r="A26" s="11" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="17" x14ac:dyDescent="0.25">
+      <c r="A28" s="12" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" ht="17" x14ac:dyDescent="0.25">
+      <c r="A30" s="12" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" ht="17" x14ac:dyDescent="0.25">
+      <c r="A31" s="12" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" ht="17" x14ac:dyDescent="0.25">
+      <c r="A32" s="12" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" ht="17" x14ac:dyDescent="0.25">
+      <c r="A34" s="12" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" ht="17" x14ac:dyDescent="0.25">
+      <c r="A35" s="12" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" ht="17" x14ac:dyDescent="0.25">
+      <c r="A36" s="12" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" ht="17" x14ac:dyDescent="0.25">
+      <c r="A38" s="12" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" ht="17" x14ac:dyDescent="0.25">
+      <c r="A39" s="12" t="s">
+        <v>215</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>